<commit_message>
style: some improvement to the template
</commit_message>
<xml_diff>
--- a/consolidador_v2/templates/conciliation_report.xlsx
+++ b/consolidador_v2/templates/conciliation_report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\projects\scraper\consolidador_v2\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B98651B4-B8AD-42D9-9F09-DFB307D450A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9E2ACAB-7E4F-40D3-9275-3086039A8F6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="330" windowWidth="24240" windowHeight="13290" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12000" yWindow="450" windowWidth="12000" windowHeight="13050" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="21" r:id="rId1"/>
@@ -3604,15 +3604,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>352425</xdr:colOff>
+      <xdr:colOff>49866</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>165866</xdr:rowOff>
+      <xdr:rowOff>143454</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>931068</xdr:colOff>
+      <xdr:colOff>628509</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
+      <xdr:rowOff>72838</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3640,8 +3640,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="1047750" y="165866"/>
-          <a:ext cx="581025" cy="500884"/>
+          <a:off x="1103219" y="143454"/>
+          <a:ext cx="578643" cy="500884"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3657,11 +3657,11 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>180975</xdr:colOff>
+      <xdr:colOff>571500</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>157380</xdr:rowOff>
+      <xdr:rowOff>168088</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1628775" cy="471270"/>
+    <xdr:ext cx="1238250" cy="460562"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="9" name="2 Imagen" descr="C:\Users\AuditoriaInterna\Desktop\SEDEMAT  ADMINISTRACIÓN\sedemat BNP\IMG-20180606-WA0006.jpg">
@@ -3688,8 +3688,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="5295900" y="157380"/>
-          <a:ext cx="1628775" cy="471270"/>
+          <a:off x="6443382" y="168088"/>
+          <a:ext cx="1238250" cy="460562"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6543,7 +6543,7 @@
       <c r="H14" s="70"/>
       <c r="J14" s="90"/>
     </row>
-    <row r="15" spans="1:12">
+    <row r="15" spans="1:12" ht="15.75" customHeight="1">
       <c r="A15" s="202" t="s">
         <v>46</v>
       </c>
@@ -6555,7 +6555,7 @@
       <c r="G15" s="204"/>
       <c r="H15" s="2"/>
     </row>
-    <row r="16" spans="1:12">
+    <row r="16" spans="1:12" ht="15.75" customHeight="1">
       <c r="A16" s="205" t="s">
         <v>21</v>
       </c>
@@ -6575,7 +6575,7 @@
       <c r="K16" s="3"/>
       <c r="L16" s="4"/>
     </row>
-    <row r="17" spans="1:17">
+    <row r="17" spans="1:17" ht="15.75" customHeight="1">
       <c r="A17" s="213"/>
       <c r="B17" s="103"/>
       <c r="C17" s="108"/>
@@ -6587,7 +6587,7 @@
       <c r="K17" s="3"/>
       <c r="L17" s="4"/>
     </row>
-    <row r="18" spans="1:17" ht="15.75">
+    <row r="18" spans="1:17" ht="15.75" customHeight="1">
       <c r="A18" s="230"/>
       <c r="B18" s="231"/>
       <c r="C18" s="231"/>
@@ -6601,7 +6601,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:17">
+    <row r="19" spans="1:17" ht="15.75" customHeight="1">
       <c r="A19" s="235"/>
       <c r="B19" s="234"/>
       <c r="C19" s="240"/>
@@ -6613,7 +6613,7 @@
       <c r="G19" s="236"/>
       <c r="H19" s="1"/>
     </row>
-    <row r="20" spans="1:17">
+    <row r="20" spans="1:17" ht="15.75" customHeight="1">
       <c r="A20" s="233" t="s">
         <v>21</v>
       </c>
@@ -6631,7 +6631,7 @@
       </c>
       <c r="H20" s="1"/>
     </row>
-    <row r="21" spans="1:17">
+    <row r="21" spans="1:17" ht="15.75" customHeight="1">
       <c r="A21" s="209"/>
       <c r="B21" s="81"/>
       <c r="C21" s="241" t="s">
@@ -6645,7 +6645,7 @@
       </c>
       <c r="H21" s="1"/>
     </row>
-    <row r="22" spans="1:17">
+    <row r="22" spans="1:17" ht="15.75" customHeight="1">
       <c r="A22" s="209"/>
       <c r="B22" s="81"/>
       <c r="C22" s="108" t="s">
@@ -6659,7 +6659,7 @@
       </c>
       <c r="H22" s="1"/>
     </row>
-    <row r="23" spans="1:17">
+    <row r="23" spans="1:17" ht="15.75" customHeight="1">
       <c r="A23" s="209"/>
       <c r="B23" s="81"/>
       <c r="C23" s="108" t="s">
@@ -6673,7 +6673,7 @@
       </c>
       <c r="H23" s="1"/>
     </row>
-    <row r="24" spans="1:17" ht="15.75">
+    <row r="24" spans="1:17" ht="15.75" customHeight="1">
       <c r="A24" s="208"/>
       <c r="B24" s="198"/>
       <c r="C24" s="198"/>
@@ -6687,7 +6687,7 @@
         <v>-103768.97</v>
       </c>
     </row>
-    <row r="25" spans="1:17">
+    <row r="25" spans="1:17" ht="15.75" customHeight="1">
       <c r="A25" s="237" t="s">
         <v>40</v>
       </c>
@@ -6702,7 +6702,7 @@
       </c>
       <c r="G25" s="211"/>
     </row>
-    <row r="26" spans="1:17">
+    <row r="26" spans="1:17" ht="15.75" customHeight="1">
       <c r="A26" s="212"/>
       <c r="B26" s="200"/>
       <c r="C26" s="200"/>
@@ -6711,7 +6711,7 @@
       <c r="F26" s="76"/>
       <c r="G26" s="211"/>
     </row>
-    <row r="27" spans="1:17">
+    <row r="27" spans="1:17" ht="15.75" customHeight="1">
       <c r="A27" s="218" t="s">
         <v>48</v>
       </c>
@@ -6728,7 +6728,7 @@
       </c>
       <c r="G27" s="211"/>
     </row>
-    <row r="28" spans="1:17">
+    <row r="28" spans="1:17" ht="15.75" customHeight="1">
       <c r="A28" s="219" t="s">
         <v>54</v>
       </c>
@@ -6748,7 +6748,7 @@
       <c r="P28" s="169"/>
       <c r="Q28" s="1"/>
     </row>
-    <row r="29" spans="1:17" ht="29.25" customHeight="1">
+    <row r="29" spans="1:17" ht="15.75" customHeight="1">
       <c r="A29" s="220"/>
       <c r="B29" s="214"/>
       <c r="C29" s="214"/>
@@ -6771,7 +6771,7 @@
       <c r="N29" s="169"/>
       <c r="O29" s="1"/>
     </row>
-    <row r="30" spans="1:17" ht="29.25" customHeight="1">
+    <row r="30" spans="1:17" ht="15.75" customHeight="1">
       <c r="A30" s="224" t="s">
         <v>56</v>
       </c>
@@ -6782,7 +6782,7 @@
       <c r="F30" s="225"/>
       <c r="G30" s="226"/>
     </row>
-    <row r="31" spans="1:17" ht="16.5" customHeight="1" thickBot="1">
+    <row r="31" spans="1:17" ht="15.75" customHeight="1" thickBot="1">
       <c r="A31" s="221" t="s">
         <v>57</v>
       </c>

</xml_diff>